<commit_message>
App web, sem resoluções e dados no formato da plataforma
- upq/web.py + upq/web/app.html: app local (biblioteca padrão) com a tela
  Enviar lista (arrastar PDFs, etapas do processamento) e a tela Listas
  (tabela → questões → detalhe no formato da plataforma, com o recorte
  original); --demo gera um HTML único com as listas embutidas
- Resolução removida do fluxo: prompt, modelo, validação, revisão, envio e
  exemplo; esforço padrão da transcrição passa a ser low
- Assuntos por questão (da base de tópicos), nome/descrição/tags da lista e
  dificuldade por extenso; migração 005 e importar_lista atualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TqB9WU1gptZGxvbH3cp7L3
</commit_message>
<xml_diff>
--- a/exemplos/Movimento_Circular_Uniforme/Movimento_Circular_Uniforme.xlsx
+++ b/exemplos/Movimento_Circular_Uniforme/Movimento_Circular_Uniforme.xlsx
@@ -585,14 +585,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>A grandeza expressa em rpm é a frequência de rotação. No SI, a frequência é medida em hertz ($1\ \text{Hz} = 1$ rotação por segundo), então basta converter minutos em segundos.
-$$f = \frac{3000\ \text{rotações}}{60\ \text{s}} = 50\ \text{Hz}$$
-As alternativas A e D tratam do período, que seria $T = \frac{1}{50} = 0{,}02\ \text{s}$; a B confunde frequência com velocidade angular ($\omega = 2\pi f = 100\pi\ \text{rad/s}$); a E multiplica por 60 em vez de dividir.
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -662,16 +655,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>A aceleração centrípeta é sempre perpendicular ao vetor velocidade e aponta para o centro da curva. Por ser perpendicular, ela não tem componente na direção do movimento: muda apenas a direção de $\vec{v}$, nunca o seu módulo. Quem altera o módulo é a aceleração tangencial.
-$$a_c = \frac{v^2}{R}$$
-- A e B: aumentar ou diminuir o módulo da velocidade é papel da aceleração tangencial.
-- D: a aceleração centrípeta não altera a magnitude de $\vec{v}$.
-- E: em movimentos retilíneos não há aceleração centrípeta.
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -742,17 +726,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>Um movimento de rotação em torno de um eixo é descrito pela velocidade angular $\omega$, que indica o ângulo descrito por unidade de tempo. Para o observador externo, manter o giro significa manter o corpo girando com velocidade angular (não nula) em torno do eixo.
-$$\omega = \frac{\Delta\varphi}{\Delta t}$$
-- A: massa é grandeza escalar; não existe “massa vetorial”.
-- B: força centrífuga só aparece para um observador no referencial que gira (não inercial), não para o observador externo.
-- C: não há mola ou deformação elástica relevante descrita.
-- E: temperatura não é grandeza cinemática do movimento.
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -818,16 +792,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>Em movimento circular uniforme, a Lua percorre uma circunferência inteira ($2\pi R$) em um período $T$.
-$$v = \frac{2\pi R}{T} = \frac{2 \cdot 3 \cdot 4{,}0 \times 10^{8}}{2{,}4 \times 10^{6}}\ \text{m/s} = \frac{24 \times 10^{8}}{2{,}4 \times 10^{6}}\ \text{m/s} = 1.000\ \text{m/s}$$
-Convertendo para km/h (multiplica por $3{,}6$):
-$$v = 1.000 \cdot 3{,}6 = 3.600\ \text{km/h}$$
-A alternativa B traz o valor numérico em m/s, mas com a unidade errada.
-**Gabarito: A**</t>
-        </is>
-      </c>
+      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -893,13 +858,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>O período é o tempo de uma volta completa. Como o comprimento da pista já é o perímetro da circunferência, basta dividir a distância de uma volta pela velocidade escalar.
-$$T = \frac{2\pi R}{v} = \frac{4.200\ \text{m}}{35\ \text{m/s}} = 120\ \text{s}$$
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -965,14 +924,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>No MCU, a velocidade escalar é o comprimento da órbita dividido pelo período. É preciso converter o período para segundos: $T = 2{,}0\ \text{h} = 7.200\ \text{s}$.
-$$v = \frac{2\pi r}{T} = \frac{2 \cdot 3{,}0 \cdot 1{,}848 \times 10^{6}\ \text{m}}{7.200\ \text{s}} = \frac{11{,}088 \times 10^{6}\ \text{m}}{7.200\ \text{s}} = 1.540\ \text{m/s}$$
-A alternativa A corresponde a $\frac{r}{T}$, esquecendo o fator $2\pi$; C e D trazem valores em km/s muito acima do correto ($1{,}54\ \text{km/s}$).
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1043,15 +995,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>Um satélite geoestacionário acompanha a rotação da Terra: ele completa uma volta em torno do eixo terrestre no mesmo tempo que a Terra gira em torno de si mesma (cerca de 24 h) e mantém sempre a mesma face voltada para a Terra. Assim, o corpo do satélite gira, em relação ao Sol, uma vez por dia.
-Para que os painéis fiquem sempre perpendiculares aos raios solares (direção praticamente fixa), eles precisam girar em relação ao satélite compensando exatamente esse giro: uma volta a cada dia, isto é, com o mesmo período da Terra.
-$$T_{\text{painéis}} = T_{\text{Terra}} \Rightarrow \omega_{\text{painéis}} = \frac{2\pi}{T_{\text{Terra}}} = R_T$$
-Valores como $0{,}5\ R_T$ ou $2\ R_T$ fariam os painéis se adiantarem ou se atrasarem em relação ao Sol ao longo do dia.
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1117,14 +1061,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>A velocidade linear de um ponto em MCU é $v = 2\pi R f$. É preciso converter a frequência para hertz e o raio para metros (a capacidade de $16\ \text{kg}$ não interfere).
-$$f = \frac{720}{60\ \text{s}} = 12\ \text{Hz} \qquad R = 50\ \text{cm} = 0{,}5\ \text{m}$$
-$$v = 2\pi R f = 2 \cdot 3 \cdot 0{,}5 \cdot 12 = 36{,}0\ \text{m/s}$$
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1190,13 +1127,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>O ponteiro dos minutos dá uma volta completa a cada hora, logo seu período é $T = 1\ \text{h} = 3.600\ \text{s}$. O raio é $R = 10\ \text{cm} = 0{,}1\ \text{m}$.
-$$v = \frac{2\pi R}{T} = \frac{2\pi \cdot 0{,}1\ \text{m}}{3.600\ \text{s}} = \frac{0{,}2\pi}{3.600} = \frac{\pi}{18000}\ \text{m/s}$$
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1269,16 +1200,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>No MCU, as grandezas se relacionam por $v = \omega r$, $a_c = \frac{v^2}{r}$ e $T = \frac{2\pi}{\omega}$. Primeiro, converta a velocidade para o SI: $v = 36\ \text{km/h} = \frac{36}{3{,}6} = 10\ \text{m/s}$.
-$$\omega = \frac{v}{r} = \frac{10\ \text{m/s}}{4\ \text{m}} = 2{,}5\ \text{rad/s}$$
-$$a_c = \frac{v^2}{r} = \frac{(10\ \text{m/s})^2}{4\ \text{m}} = 25\ \text{m/s}^2$$
-$$T = \frac{2\pi}{\omega} = \frac{2 \cdot 3{,}14}{2{,}5\ \text{rad/s}} \approx 2{,}5\ \text{s}$$
-A alternativa A tem o $\omega$ correto, mas erra a aceleração e o período; as demais não satisfazem as relações do MCU com os dados fornecidos.
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1346,16 +1268,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>A cada salto a corda dá uma volta completa, então o número de saltos por segundo é a frequência do movimento circular do ponto P. A velocidade escalar é $v = 2\pi r f$.
-Frequência:
-$$f = \frac{105}{30\ \text{s}} = 3{,}5\ \text{Hz}$$
-Velocidade, com $r = 0{,}9\ \text{m}$:
-$$v = 2\pi r f = 2 \cdot 3 \cdot 0{,}9 \cdot 3{,}5 = 18{,}9\ \text{m/s}$$
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1426,17 +1339,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>Sem deslizamento, a velocidade do carro é igual à velocidade linear dos pontos da borda do pneu: $v = 2\pi R f$. Basta isolar a frequência e convertê-la para rpm.
-Dados no SI: $v = 90\ \text{km/h} = 25\ \text{m/s}$ e $R = \frac{625}{2}\ \text{mm} = 0{,}3125\ \text{m}$.
-$$f = \frac{v}{2\pi R} = \frac{25}{2 \cdot 3{,}0 \cdot 0{,}3125} = \frac{25}{1{,}875} \approx 13{,}3\ \text{Hz}$$
-Em rotações por minuto:
-$$f = 13{,}3 \cdot 60 \approx 800\ \text{rpm}$$
-O valor está na faixa entre $751$ e $800$ rpm.
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1509,17 +1412,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>No movimento circular, a aceleração centrípeta é responsável apenas pela mudança de direção da velocidade; ela tem a direção do raio e aponta para o centro da trajetória, com módulo $a_c = \frac{v^2}{R} = \omega^2 R$.
-- **A — Incorreta.** A variação da velocidade (em módulo) por unidade de tempo é a aceleração tangencial; a centrípeta está ligada à mudança de direção.
-- **B — Incorreta.** A frequência é o número de voltas por unidade de tempo, não o total de voltas ao final do processo.
-- **C — Incorreta.** O período é o tempo de uma volta completa, não o tempo total da extração.
-- **D — Incorreta.** A aceleração centrípeta é radial (perpendicular à velocidade), não tangente.
-- **E — Correta.** A aceleração centrípeta tem a direção do raio do tambor, apontando para o centro.
-**Gabarito: E**</t>
-        </is>
-      </c>
+      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1589,14 +1482,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>Rodando sem deslizar, a cadeira avança com a mesma velocidade linear dos pontos da borda da roda: $v = 2\pi R f$.
-Com $R = 30\ \text{cm} = 0{,}3\ \text{m}$ e $f = 5\ \text{Hz}$:
-$$v = 2\pi \cdot 0{,}3 \cdot 5 = 3\pi \approx 3 \cdot 3{,}14 \approx 9{,}4\ \text{m/s}$$
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1662,16 +1548,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>No MCU a velocidade escalar é constante, então ela sai da distância percorrida no intervalo. Depois, o período vem de $v = \frac{2\pi R}{T}$.
-Velocidade escalar:
-$$v = \frac{\Delta s}{\Delta t} = \frac{108\ \text{m}}{(5 - 2)\ \text{s}} = 36\ \text{m/s}$$
-Período:
-$$T = \frac{2\pi R}{v} = \frac{2\pi \cdot 6}{36} = \frac{\pi}{3}\ \text{s}$$
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1740,16 +1617,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>O ponto P descreve uma circunferência de raio $R = 60\ \text{cm}$ (dado na figura). Sua velocidade linear é $v = 2\pi R f$, com a frequência em hertz.
-Conversão da frequência:
-$$f = \frac{300\ \text{rpm}}{60} = 5\ \text{Hz}$$
-Velocidade do ponto P, com $R = 0{,}6\ \text{m}$:
-$$v = 2\pi R f = 2 \cdot 3 \cdot 0{,}6 \cdot 5 = 18\ \text{m/s}$$
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1816,18 +1684,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>Após soltar o cordão, cada objeto faz um lançamento horizontal a partir da mesma altura. O tempo de queda depende só da altura, $t = \sqrt{\frac{2h}{g}}$, e não da massa; o alcance é $A = v_x \cdot t$.
-Como os dois caem da mesma altura (mesmo $t$) e atingem o mesmo ponto (mesmo $A$):
-$$v_{x,1} = \frac{A}{t} = v_{x,2}$$
-- **A — Incorreta.** Mesma velocidade tangencial e mesmo raio (mesmo cordão) dão a mesma velocidade angular, $\omega = \frac{v}{R}$.
-- **B — Incorreta.** O tempo de queda independe da massa; os dois levam o mesmo tempo.
-- **C — Correta.** Mesmo tempo de queda e mesmo alcance implicam a mesma velocidade horizontal.
-- **D — Incorreta.** $F_c = \frac{m v^2}{R}$: com mesmos $v$ e $R$, a força sobre o objeto 2 é o dobro da do objeto 1.
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1897,16 +1754,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="O19" s="2" t="inlineStr">
-        <is>
-          <t>O velocímetro mede a frequência $f$ das rodas e calcula $v = 2\pi R f$ usando o raio para o qual foi calibrado ($30\ \text{cm}$). A frequência real é a mesma; o que muda é o raio verdadeiro ($27\ \text{cm}$).
-Frequência que gera a indicação de $90\ \text{km/h}$:
-$$90 = 2\pi \cdot 0{,}30 \cdot f$$
-Velocidade real, com a mesma $f$:
-$$v_{\text{real}} = 2\pi \cdot 0{,}27 \cdot f = 90 \cdot \frac{0{,}27}{0{,}30} = 90 \cdot 0{,}9 = 81\ \text{km/h}$$
-**Gabarito: C**</t>
-        </is>
-      </c>
+      <c r="O19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1975,14 +1823,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O20" s="2" t="inlineStr">
-        <is>
-          <t>As amostras periféricas descrevem uma circunferência de raio $R = 0{,}15\ \text{m}$ com frequência $f = 60\ \text{Hz}$. A velocidade linear é $v = 2\pi R f$.
-$$v = 2\pi \cdot 0{,}15 \cdot 60 = 18\pi \approx 18 \cdot 3{,}14 \approx 56{,}5\ \text{m/s}$$
-O valor mais próximo é $57\ \text{m/s}$.
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2058,20 +1899,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O21" s="2" t="inlineStr">
-        <is>
-          <t>Em MCU a velocidade tem módulo constante e a aceleração é só centrípeta, $a_c = \frac{v^2}{R}$, voltada para o centro. Dados: $v = 72\ \text{km/h} = 20\ \text{m/s}$ e $R = 100\ \text{m}$.
-**I. Verdadeira.**
-$$a_c = \frac{v^2}{R} = \frac{20^2}{100} = 4\ \text{m/s}^2$$
-**II. Verdadeira.** A aceleração centrípeta é radial e aponta para o centro da curva.
-**III. Falsa.** Ao completar uma volta o carro retorna ao ponto de partida: o deslocamento é nulo. (A distância percorrida seria $2\pi R \approx 628\ \text{m}$, não $200\ \text{m}$.)
-**IV. Verdadeira.** Numa rotatória plana, a resultante centrípeta é dada pelo atrito lateral entre os pneus e o asfalto.
-**V. Falsa.**
-$$T = \frac{2\pi R}{v} = \frac{2\pi \cdot 100}{20} = 10\pi \approx 31{,}4\ \text{s}$$
-São verdadeiras apenas I, II e IV.
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2139,15 +1967,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O22" s="2" t="inlineStr">
-        <is>
-          <t>Para haver sincronismo, a cada flash da lâmpada o parafuso deve estar de novo na posição da seta, ou seja, ele dá uma volta completa a cada intervalo entre flashes. Assim, a frequência de rotação do disco é igual à frequência da luz.
-$$f = 2\ \text{kHz} = 2 \times 10^{3}\ \text{Hz}$$
-A velocidade escalar de um ponto da periferia é:
-$$v = 2\pi R f = 2 \cdot 3{,}14 \cdot 1 \cdot 2 \times 10^{3} \approx 12{,}56 \times 10^{3}\ \text{m/s}$$
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2224,21 +2044,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
-        <is>
-          <t>No movimento circular uniforme, a velocidade linear relaciona-se com a angular por $v = \omega R$, e a frequência por $\omega = 2\pi f$.
-Convertendo a velocidade:
-$$v = 36\ \text{km/h} = \frac{36}{3{,}6} = 10\ \text{m/s}$$
-**I. Verdadeira.**
-$$\omega = \frac{v}{R} = \frac{10}{20} = 0{,}5\ \text{rad/s}$$
-**II. Verdadeira.**
-$$f = \frac{\omega}{2\pi} = \frac{0{,}5}{2 \cdot 3} = \frac{1}{12}\ \text{Hz}$$
-**III. Verdadeira.** O comprimento da rotatória é
-$$C = 2\pi R = 2 \cdot 3 \cdot 20 = 120\ \text{m}$$
-e $\frac{420}{120} = 3{,}5$.
-**Gabarito: E**</t>
-        </is>
-      </c>
+      <c r="O23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2304,19 +2110,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O24" s="2" t="inlineStr">
-        <is>
-          <t>Como as pistas são concêntricas, o alinhamento depende só das velocidades angulares. O carrinho mais rápido (em ângulo) ganha uma volta sobre o outro a cada alinhamento, com velocidade angular relativa constante.
-Velocidades angulares:
-$$\omega_{NP} = \frac{V}{R} \qquad \omega_{AS} = \frac{2V}{1{,}5R} = \frac{4V}{3R}$$
-Velocidade angular relativa:
-$$\omega_{\text{rel}} = \frac{4V}{3R} - \frac{V}{R} = \frac{V}{3R}$$
-Entre dois alinhamentos consecutivos o ângulo relativo varia $2\pi$, e isso leva sempre o mesmo tempo:
-$$\Delta t = \frac{2\pi}{\omega_{\text{rel}}} = 2\ \text{s}$$
-Logo, os alinhamentos ocorrem em $t = 2\ \text{s}$, $4\ \text{s}$ e $6\ \text{s}$. O terceiro reencontro ocorre em $t = 6\ \text{s}$.
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2386,16 +2180,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
-        <is>
-          <t>No movimento circular uniforme a aceleração é apenas a centrípeta, $a_{cp} = \omega^2 R$, com $\omega = \frac{2\pi}{T}$.
-$$\omega = \frac{2\pi}{T} = \frac{2 \cdot 3{,}0}{3{,}0} = 2\ \text{rad/s}$$
-$$a_{cp} = \omega^2 R = 2^2 \cdot 5{,}0 = 20\ \text{m/s}^2$$
-Comparando com $g$:
-$$\frac{a_{cp}}{g} = \frac{20}{10} = 2 \Rightarrow a_{cp} = 2g$$
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2467,16 +2252,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="O26" s="2" t="inlineStr">
-        <is>
-          <t>Correndo em sentidos opostos, as velocidades angulares se somam no movimento relativo. Entre dois encontros, juntos eles completam uma volta ($2\pi$), então as frequências se somam:
-$$\frac{1}{T_{B}} + \frac{1}{T_{V}} = \frac{1}{T_{\text{enc}}}$$
-$$\frac{1}{48} + \frac{1}{T_{V}} = \frac{1}{18}$$
-$$\frac{1}{T_{V}} = \frac{1}{18} - \frac{1}{48} = \frac{8 - 3}{144} = \frac{5}{144}$$
-$$T_{V} = \frac{144}{5} = 28{,}8\ \text{s}$$
-**Gabarito: A**</t>
-        </is>
-      </c>
+      <c r="O26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2542,16 +2318,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr">
-        <is>
-          <t>Na curva, a resultante central é a força centrípeta, $F = \frac{mV^2}{R}$.
-Situação inicial e nova situação (velocidade $2V$, força $\frac{F}{2}$, raio $R'$):
-$$F = \frac{mV^2}{R} \qquad \frac{F}{2} = \frac{m(2V)^2}{R'} = \frac{4mV^2}{R'}$$
-Dividindo a segunda pela primeira:
-$$\frac{1}{2} = \frac{4R}{R'} \Rightarrow R' = 8R$$
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2621,18 +2388,7 @@
           <t>E</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>No movimento circular, as velocidades angular e tangencial (linear) estão ligadas pelo raio da trajetória:
-$$v = \omega R$$
-Portanto elas **não** são independentes: para um mesmo raio, dobrar $\omega$ dobra $v$. A alternativa E é a incorreta.
-- A: correta. A tração na corda puxa a madeira para o centro, isto é, para a mão do curumim.
-- B: correta. O peso é sempre vertical, apontando para o centro da Terra.
-- C: correta. Ao soltar a corda, a madeira sai pela tangente com a velocidade tangencial que tinha, e o alcance depende dela.
-- D: correta. Sem resultante centrípeta não há mudança de direção da velocidade, e o corpo seguiria em linha reta.
-**Gabarito: E**</t>
-        </is>
-      </c>
+      <c r="O28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2699,18 +2455,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O29" s="2" t="inlineStr">
-        <is>
-          <t>O satélite geoestacionário e o ponto do Equador têm o mesmo período ($T = 24\ \text{h}$), logo a mesma velocidade angular. Então a velocidade tangencial é proporcional ao raio: $v = \omega r$.
-Raio da Terra, a partir da velocidade do ponto no Equador:
-$$v_T = \frac{2\pi R_T}{T} \Rightarrow R_T = \frac{v_T\, T}{2\pi} = \frac{1600 \cdot 24}{2 \cdot 3} = 6400\ \text{km}$$
-Raio da órbita do satélite:
-$$r = R_T + h = 6400 + 36000 = 42400\ \text{km}$$
-Com a mesma $\omega$:
-$$\frac{v_S}{v_T} = \frac{r}{R_T} \Rightarrow v_S = 1600 \cdot \frac{42400}{6400} = 10600\ \text{km/h}$$
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2789,20 +2534,7 @@
           <t>D</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr">
-        <is>
-          <t>Na curva horizontal, a componente vertical da sustentação equilibra o peso e a componente horizontal faz o papel de resultante centrípeta. Com $m = 2000\ \text{kg}$:
-$$F\cos 45^\circ = mg \qquad F\,\text{sen}\,45^\circ = F_{cp}$$
-Dividindo uma pela outra:
-$$F_{cp} = mg \tan 45^\circ = 2000 \cdot 10 \cdot 1 = 20000\ \text{N} = 20\ \text{kN}$$
-E, como $F_{cp} = \frac{mv^2}{R}$:
-$$\frac{mv^2}{R} = mg\tan 45^\circ \Rightarrow v^2 = gR = 10 \cdot 1000 = 10000 \Rightarrow v = 100\ \text{m/s} = 360\ \text{km/h}$$
-**I. Falsa.** O avião faz curva, então a resultante é centrípeta e não nula.
-**II. Verdadeira.** $F_{cp} = 20\ \text{kN}$.
-**III. Verdadeira.** $v = 100\ \text{m/s} = 360\ \text{km/h}$.
-**Gabarito: D**</t>
-        </is>
-      </c>
+      <c r="O30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2870,19 +2602,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="O31" s="2" t="inlineStr">
-        <is>
-          <t>No MCU a resultante centrípeta tem o mesmo módulo em todos os pontos, $F_{cp} = \frac{mv^2}{R}$, sempre apontando para o centro. O veículo percorre o trilho por dentro, então a normal aponta para o centro.
-**Posição 1 (ponto mais baixo):** normal para cima (centro), peso para baixo.
-$$N_1 - mg = \frac{mv^2}{R} \Rightarrow N_1 = \frac{mv^2}{R} + mg$$
-**Posição 3 (ponto mais alto):** normal e peso para baixo (centro).
-$$N_3 + mg = \frac{mv^2}{R} \Rightarrow N_3 = \frac{mv^2}{R} - mg$$
-**Posições 2 e 4 (horizontal):** o peso é perpendicular ao raio e só a normal é centrípeta.
-$$N_2 = N_4 = \frac{mv^2}{R}$$
-Portanto $N_1 &gt; N_2 = N_4 &gt; N_3$, o que confirma $N_1 &gt; N_3$ e $N_4 = N_2$.
-**Gabarito: B**</t>
-        </is>
-      </c>
+      <c r="O31" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>